<commit_message>
Generated output file from workflow
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -498,6 +498,581 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FMCC - PCKG 22 UPDATE: WORK STILL NEED TO BE COMP...</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CATHEDRAL AVE NW</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Update-Renewal</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26812239</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>26748362</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>10/23/26 12:34 pm</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>10/27/26 12:45 pm</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>11/16/26 12:45 pm</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>COMDC, VDC, WASA02 &amp; WGL07 - Not yet responded &amp; DCDOT01 - Not complete/In progress</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>21 days, 21:47:50.948360</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FMCC - PCKG 20</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DOUGLAS ST NE</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26811942</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>10/23/26 11:25 am</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>10/28/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>11/16/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>COMDC, WASA02 &amp; WGL07 - Not yet responded &amp; DCDOT01 - Not complete/In progress</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>21 days, 20:32:50.948289</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FMCC - PCKG 20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>22ND ST NE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26811941</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>10/23/26 11:25 am</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>10/28/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>11/16/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>DCDOT01 - Not complete/In progress &amp; VDC, WASA02 &amp; WGL07 - Not yet responded</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>21 days, 20:32:50.948235</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>FMCC - PCKG 20</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>24TH ST NE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26811940</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>10/23/26 11:25 am</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>10/28/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>11/16/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>DCDOT01 - Not complete/In progress &amp; VDC, WASA02 &amp; WGL07 - Not yet responded</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>21 days, 20:32:50.948193</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FMCC - PCKG 20</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>24TH ST NE</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26811939</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>10/23/26 11:25 am</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>10/28/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>11/16/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>DCDOT01 - Not complete/In progress &amp; VDC, WASA02 &amp; WGL07 - Not yet responded</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>21 days, 20:32:50.948155</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FMCC - PCKG 20</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>22ND ST NE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26811938</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>10/23/26 11:25 am</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>10/28/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>11/16/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>DCDOT01 - Not complete/In progress &amp; VDC, WASA02 &amp; WGL07 - Not yet responded</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>21 days, 20:32:50.948071</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FMCC - PCKG 20</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DOUGLAS ST NE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26811937</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>10/23/26 11:25 am</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>10/28/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>11/16/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>DCDOT01 - Not complete/In progress &amp; VDC, WASA02 &amp; WGL07 - Not yet responded</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>21 days, 20:32:50.948026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>FMCC - PCKG 20</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>22ND ST NE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26811936</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>10/23/26 11:25 am</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>10/28/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>11/16/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>DCDOT01 - Not complete/In progress &amp; VDC, WASA02 &amp; WGL07 - Not yet responded</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>21 days, 20:32:50.947988</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FMMC - PCKG 20</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>22ND ST NE</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26811935</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>10/23/26 11:25 am</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>10/28/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>11/16/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>DCDOT01 - Not complete/In progress &amp; VDC, WASA02 &amp; WGL07 - Not yet responded</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>21 days, 20:32:50.947952</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FMCC - PCKG 20</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>24TH ST NE</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 26811934</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>10/23/26 11:25 am</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>10/28/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>11/16/26 11:30 am</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>COMDC, VDC, WASA02 &amp; WGL07 - Not yet responded &amp; DCDOT01 - Not complete/In progress</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>21 days, 20:32:50.947913</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>